<commit_message>
feat(105): Agregado de columnas en plantilla de crecimientos
</commit_message>
<xml_diff>
--- a/templates/template_import_data_weighings.xlsx
+++ b/templates/template_import_data_weighings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jesus\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F466F0D-EA25-464E-9314-520B3F9A89DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431E0E87-0C76-4DF9-BCF4-30FAAA06FD51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PesosCorporales" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Único</t>
   </si>
@@ -58,6 +58,12 @@
   </si>
   <si>
     <t>Tipo pesaje</t>
+  </si>
+  <si>
+    <t>Razón de Eliminación</t>
+  </si>
+  <si>
+    <t>Comentario de Eliminación</t>
   </si>
 </sst>
 </file>
@@ -127,7 +133,13 @@
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="14">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
@@ -192,20 +204,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Animales" displayName="Animales" ref="A1:K11" totalsRowShown="0" headerRowDxfId="11">
-  <autoFilter ref="A1:K11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Único" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="ID Electrónico" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Práctico" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Tipo pesaje" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Peso" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Altura" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Condición" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Técnico" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Comentario" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Lote" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Animales" displayName="Animales" ref="A1:M11" totalsRowShown="0" headerRowDxfId="13">
+  <autoFilter ref="A1:M11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Único" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="ID Electrónico" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Práctico" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Tipo pesaje" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{776F9392-8934-43CC-8E6C-7C552F1BA4C0}" name="Razón de Eliminación" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{D59B66F7-6BE4-469C-8B54-F8BEFE3BEA91}" name="Comentario de Eliminación" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Peso" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Altura" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Condición" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Técnico" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Comentario" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Lote" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -474,21 +488,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="12.5703125" customWidth="1"/>
     <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" customWidth="1"/>
-    <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.28515625" customWidth="1"/>
-    <col min="10" max="10" width="16.85546875" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.28515625" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" customWidth="1"/>
+    <col min="13" max="13" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -505,155 +521,181 @@
         <v>10</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="6"/>
       <c r="K2" s="3"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="2"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="6"/>
       <c r="K3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="2"/>
       <c r="E4" s="3"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="6"/>
       <c r="K4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="2"/>
       <c r="E5" s="3"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="6"/>
       <c r="K5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="2"/>
       <c r="E6" s="3"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="6"/>
       <c r="K6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="2"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="6"/>
       <c r="K7" s="3"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="2"/>
       <c r="E8" s="3"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="6"/>
       <c r="K8" s="3"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="2"/>
       <c r="E9" s="3"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="6"/>
       <c r="K9" s="3"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="2"/>
       <c r="E10" s="3"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="6"/>
       <c r="K10" s="3"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="2"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="6"/>
       <c r="K11" s="3"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -661,15 +703,20 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
-      <c r="H12" s="2"/>
+      <c r="H12" s="3"/>
       <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
+      <c r="J12" s="2"/>
       <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E11" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"General,Al nacer,Al ingreso,Al destete,Al servicio,Al parto,Al secado,Al salir"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F11" xr:uid="{D3CA9356-0153-4450-9B63-DC3AD77F0E03}">
+      <formula1>"Venta,Muerte,Egreso"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Merged PR 1172: Agregado de columnas en plantilla de crecimientos
feat(105): Agregado de columnas en plantilla de crecimientos

Related work items: #105
</commit_message>
<xml_diff>
--- a/templates/template_import_data_weighings.xlsx
+++ b/templates/template_import_data_weighings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jesus\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F466F0D-EA25-464E-9314-520B3F9A89DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431E0E87-0C76-4DF9-BCF4-30FAAA06FD51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PesosCorporales" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Único</t>
   </si>
@@ -58,6 +58,12 @@
   </si>
   <si>
     <t>Tipo pesaje</t>
+  </si>
+  <si>
+    <t>Razón de Eliminación</t>
+  </si>
+  <si>
+    <t>Comentario de Eliminación</t>
   </si>
 </sst>
 </file>
@@ -127,7 +133,13 @@
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="14">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
@@ -192,20 +204,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Animales" displayName="Animales" ref="A1:K11" totalsRowShown="0" headerRowDxfId="11">
-  <autoFilter ref="A1:K11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Único" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="ID Electrónico" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Práctico" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Tipo pesaje" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Peso" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Altura" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Condición" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Técnico" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Comentario" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Lote" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Animales" displayName="Animales" ref="A1:M11" totalsRowShown="0" headerRowDxfId="13">
+  <autoFilter ref="A1:M11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Único" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="ID Electrónico" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Práctico" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Tipo pesaje" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{776F9392-8934-43CC-8E6C-7C552F1BA4C0}" name="Razón de Eliminación" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{D59B66F7-6BE4-469C-8B54-F8BEFE3BEA91}" name="Comentario de Eliminación" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Peso" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Altura" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Condición" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Técnico" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Comentario" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Lote" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -474,21 +488,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="12.5703125" customWidth="1"/>
     <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" customWidth="1"/>
-    <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.28515625" customWidth="1"/>
-    <col min="10" max="10" width="16.85546875" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.28515625" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" customWidth="1"/>
+    <col min="13" max="13" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -505,155 +521,181 @@
         <v>10</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="6"/>
       <c r="K2" s="3"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="2"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="6"/>
       <c r="K3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="2"/>
       <c r="E4" s="3"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="6"/>
       <c r="K4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="2"/>
       <c r="E5" s="3"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="6"/>
       <c r="K5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="2"/>
       <c r="E6" s="3"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="6"/>
       <c r="K6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="2"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="6"/>
       <c r="K7" s="3"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="2"/>
       <c r="E8" s="3"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="6"/>
       <c r="K8" s="3"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="2"/>
       <c r="E9" s="3"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="6"/>
       <c r="K9" s="3"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="2"/>
       <c r="E10" s="3"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="6"/>
       <c r="K10" s="3"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="2"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="6"/>
       <c r="K11" s="3"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -661,15 +703,20 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
-      <c r="H12" s="2"/>
+      <c r="H12" s="3"/>
       <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
+      <c r="J12" s="2"/>
       <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E11" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"General,Al nacer,Al ingreso,Al destete,Al servicio,Al parto,Al secado,Al salir"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F11" xr:uid="{D3CA9356-0153-4450-9B63-DC3AD77F0E03}">
+      <formula1>"Venta,Muerte,Egreso"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>